<commit_message>
Odiobuk web: one sign-in for the whole run; 17/17 green; report updated
- src/utils/odiobuk-session.ts: one admin sign-in per run, saved session
  reused by every spec. The app's httpOnly refresh cookie rotates on use,
  so closeSharedSession() writes the latest cookie back before closing
  (replaying the sign-in cookie logged the next spec out).
- home, documents, library, voices, profile, both narration E2Es: use the
  shared session; shared-account changes are undone (un-save, name restore)
- login: signs in with the shared account instead of registering two
- registration: TC-001's new account also serves TC-007 (saved.spec merged)
- admin-session.ts removed (replaced by odiobuk-session.ts)
- ListenPage: wait for the voice list to load before checking a voice
- Report: web 17/17 pass, mobile 33 pass + 2 skipped, 10 findings
</commit_message>
<xml_diff>
--- a/docs/odiobuk/Odiobuk_Test_Report.xlsx
+++ b/docs/odiobuk/Odiobuk_Test_Report.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Web Results'!$A$1:$H$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Mobile Results'!$A$1:$G$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Findings'!$A$1:$F$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Findings'!$A$1:$F$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -44,7 +44,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -69,11 +69,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
     <fill>
@@ -145,10 +140,10 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -516,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -538,7 +533,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Web: full cycle 2026-10-02 · https://odiobuk.eastus2.cloudapp.azure.com (chromium, 1 worker)</t>
+          <t>Web: full cycle 2026-10-02 · https://odiobuk.eastus2.cloudapp.azure.com (chromium, 1 worker) · ONE admin sign-in shared by the whole run; only sign-up, sign-in and the cross-account security test use their own accounts</t>
         </is>
       </c>
     </row>
@@ -603,13 +598,13 @@
         <v>17</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D7" s="5" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>0</v>
@@ -627,10 +622,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" s="7" t="n">
         <v>0</v>
@@ -684,20 +679,20 @@
         <v>1</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D10" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>100%</t>
         </is>
       </c>
     </row>
@@ -731,14 +726,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Saved</t>
+          <t xml:space="preserve">   Voices</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D12" s="7" t="n">
         <v>0</v>
@@ -758,7 +753,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Voices</t>
+          <t xml:space="preserve">   Admin · PDF catalogue</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -785,41 +780,41 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Admin · PDF catalogue</t>
+          <t xml:space="preserve">   Profile (You)</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>2</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D14" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>100%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Profile (You)</t>
+          <t xml:space="preserve">   E2E · PDF narration</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>0</v>
@@ -839,34 +834,34 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   E2E · PDF narration</t>
+          <t xml:space="preserve">   E2E · Catalogue narration</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>1</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D16" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>100%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">   E2E · Catalogue narration</t>
+          <t xml:space="preserve">   Security</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -891,54 +886,54 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Security</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>1</v>
-      </c>
-      <c r="C18" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>MOBILE</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>MOBILE</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="C19" s="4" t="n">
-        <v>33</v>
-      </c>
-      <c r="D19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Login</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
@@ -947,14 +942,14 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Login</t>
+          <t xml:space="preserve">   Registration</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C20" s="6" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D20" s="7" t="n">
         <v>0</v>
@@ -974,14 +969,14 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Registration</t>
+          <t xml:space="preserve">   Verified session</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C21" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D21" s="7" t="n">
         <v>0</v>
@@ -1001,14 +996,14 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Verified session</t>
+          <t xml:space="preserve">   Home</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C22" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D22" s="7" t="n">
         <v>0</v>
@@ -1017,7 +1012,7 @@
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1028,11 +1023,11 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Home</t>
+          <t xml:space="preserve">   Library</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C23" s="6" t="n">
         <v>4</v>
@@ -1044,7 +1039,7 @@
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1055,14 +1050,14 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Library</t>
+          <t xml:space="preserve">   Audiobooks &amp; Player</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C24" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D24" s="7" t="n">
         <v>0</v>
@@ -1082,14 +1077,14 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Audiobooks &amp; Player</t>
+          <t xml:space="preserve">   Voices</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C25" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D25" s="7" t="n">
         <v>0</v>
@@ -1109,14 +1104,14 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Voices</t>
+          <t xml:space="preserve">   Profile</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C26" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D26" s="7" t="n">
         <v>0</v>
@@ -1136,14 +1131,14 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Profile</t>
+          <t xml:space="preserve">   Vault</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C27" s="6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D27" s="7" t="n">
         <v>0</v>
@@ -1161,63 +1156,36 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Vault</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL (web + mobile)</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>52</v>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C28" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D28" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" t="inlineStr">
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL (web + mobile)</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="n">
-        <v>52</v>
-      </c>
-      <c r="C29" s="4" t="n">
-        <v>46</v>
-      </c>
-      <c r="D29" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F29" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G29" s="3" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>Findings: 8 (see the Findings sheet)</t>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Findings: 10 (see the Findings sheet)</t>
         </is>
       </c>
     </row>
@@ -1319,11 +1287,11 @@
         </is>
       </c>
       <c r="G2" s="9" t="n">
-        <v>11.1</v>
+        <v>11.2</v>
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
-          <t>Sign-up now lands on a new /welcome step ("What brings you here?"); tests skip it as a user can.</t>
+          <t>Creates the run's one new account (sign-up is the test). Sign-up now lands on a new /welcome step ("What brings you here?"), skipped as a user can.</t>
         </is>
       </c>
     </row>
@@ -1359,9 +1327,13 @@
         </is>
       </c>
       <c r="G3" s="9" t="n">
-        <v>18</v>
-      </c>
-      <c r="H3" s="9" t="inlineStr"/>
+        <v>6.1</v>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>Signs in itself (sign-in is the test), with the shared admin account — no new account.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -1395,9 +1367,13 @@
         </is>
       </c>
       <c r="G4" s="9" t="n">
-        <v>12.7</v>
-      </c>
-      <c r="H4" s="9" t="inlineStr"/>
+        <v>4.8</v>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>Wrong password for the shared admin account → "Invalid email or password", stays signed out.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -1425,17 +1401,17 @@
           <t>home.spec.ts</t>
         </is>
       </c>
-      <c r="F5" s="11" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G5" s="9" t="n">
-        <v>31</v>
+        <v>7.7</v>
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>Blocked: the admin test account (MOBILE_TEST_ADMIN_EMAIL) is rejected — UI "Invalid email or password", POST /api/auth/login → 401 (checked 2026-10-02). Needs the current admin credentials.</t>
+          <t>Shared session (the run's single admin sign-in).</t>
         </is>
       </c>
     </row>
@@ -1471,9 +1447,13 @@
         </is>
       </c>
       <c r="G6" s="9" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="H6" s="9" t="inlineStr"/>
+        <v>6.8</v>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>Shared session (the run's single admin sign-in).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -1509,7 +1489,11 @@
       <c r="G7" s="9" t="n">
         <v>5.7</v>
       </c>
-      <c r="H7" s="9" t="inlineStr"/>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>Shared session (the run's single admin sign-in).</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -1543,9 +1527,13 @@
         </is>
       </c>
       <c r="G8" s="9" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="H8" s="9" t="inlineStr"/>
+        <v>11.6</v>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>Shared session (the run's single admin sign-in). The saved title is un-saved afterwards, leaving the shared account as it was.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -1555,7 +1543,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Saved</t>
+          <t>Registration</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -1570,7 +1558,7 @@
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>saved.spec.ts</t>
+          <t>registration.spec.ts</t>
         </is>
       </c>
       <c r="F9" s="10" t="inlineStr">
@@ -1579,11 +1567,11 @@
         </is>
       </c>
       <c r="G9" s="9" t="n">
-        <v>16.6</v>
+        <v>5.6</v>
       </c>
       <c r="H9" s="9" t="inlineStr">
         <is>
-          <t>First run hit a laptop network error (DNS ERR_NAME_NOT_RESOLVED / ERR_ABORTED) at the same moment as two other tests; re-run on its own and passed.</t>
+          <t>Reuses TC-001's brand-new account (no extra sign-up).</t>
         </is>
       </c>
     </row>
@@ -1619,11 +1607,11 @@
         </is>
       </c>
       <c r="G10" s="9" t="n">
-        <v>5.1</v>
+        <v>6.7</v>
       </c>
       <c r="H10" s="9" t="inlineStr">
         <is>
-          <t>First run hit a laptop network error (DNS ERR_NAME_NOT_RESOLVED / ERR_ABORTED) at the same moment as two other tests; re-run on its own and passed.</t>
+          <t>Shared session (the run's single admin sign-in).</t>
         </is>
       </c>
     </row>
@@ -1659,11 +1647,11 @@
         </is>
       </c>
       <c r="G11" s="9" t="n">
-        <v>3.9</v>
+        <v>3.8</v>
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>Did not run in the full run (serial file stopped at TC-008's network error); passed on re-run.</t>
+          <t>Shared session (the run's single admin sign-in).</t>
         </is>
       </c>
     </row>
@@ -1693,17 +1681,17 @@
           <t>documents.spec.ts</t>
         </is>
       </c>
-      <c r="F12" s="11" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G12" s="9" t="n">
-        <v>0</v>
+        <v>5.8</v>
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>Blocked: the admin test account (MOBILE_TEST_ADMIN_EMAIL) is rejected — UI "Invalid email or password", POST /api/auth/login → 401 (checked 2026-10-02). Needs the current admin credentials.</t>
+          <t>Shared session (the run's single admin sign-in).</t>
         </is>
       </c>
     </row>
@@ -1739,9 +1727,13 @@
         </is>
       </c>
       <c r="G13" s="9" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="H13" s="9" t="inlineStr"/>
+        <v>11.8</v>
+      </c>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>Shared session (the run's single admin sign-in). The original display name is restored afterwards.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -1779,7 +1771,7 @@
       </c>
       <c r="H14" s="9" t="inlineStr">
         <is>
-          <t>Test updated: deleting now also requires the account password; "DELETE" alone keeps the button disabled.</t>
+          <t>Shared session (the run's single admin sign-in). Test updated: deleting now also requires the account password; "DELETE" alone keeps the button disabled.</t>
         </is>
       </c>
     </row>
@@ -1809,17 +1801,17 @@
           <t>narration-e2e.spec.ts</t>
         </is>
       </c>
-      <c r="F15" s="11" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G15" s="9" t="n">
-        <v>34.4</v>
+        <v>95.3</v>
       </c>
       <c r="H15" s="9" t="inlineStr">
         <is>
-          <t>Blocked: the admin test account (MOBILE_TEST_ADMIN_EMAIL) is rejected — UI "Invalid email or password", POST /api/auth/login → 401 (checked 2026-10-02). Needs the current admin credentials.</t>
+          <t>Shared session (the run's single admin sign-in). Real upload → publish → house-voice narration → done in ~1.6 min; draft title removed afterwards.</t>
         </is>
       </c>
     </row>
@@ -1849,17 +1841,17 @@
           <t>documents.spec.ts</t>
         </is>
       </c>
-      <c r="F16" s="11" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="F16" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G16" s="9" t="n">
-        <v>0</v>
+        <v>15.1</v>
       </c>
       <c r="H16" s="9" t="inlineStr">
         <is>
-          <t>Blocked: the admin test account (MOBILE_TEST_ADMIN_EMAIL) is rejected — UI "Invalid email or password", POST /api/auth/login → 401 (checked 2026-10-02). Needs the current admin credentials.</t>
+          <t>Shared session (the run's single admin sign-in). Uploaded draft title removed afterwards.</t>
         </is>
       </c>
     </row>
@@ -1895,11 +1887,11 @@
         </is>
       </c>
       <c r="G17" s="9" t="n">
-        <v>336.4</v>
+        <v>223.6</v>
       </c>
       <c r="H17" s="9" t="inlineStr">
         <is>
-          <t>Real narration of a free catalogue title with a house voice — finished in ~5.6 min.</t>
+          <t>Shared session (the run's single admin sign-in). Real narration finished in ~3.7 min. First run failed on a test timing issue (the voice list loads a moment after the select appears); fixed to wait for it, re-run alone and passed.</t>
         </is>
       </c>
     </row>
@@ -1935,11 +1927,11 @@
         </is>
       </c>
       <c r="G18" s="9" t="n">
-        <v>27.2</v>
+        <v>27</v>
       </c>
       <c r="H18" s="9" t="inlineStr">
         <is>
-          <t>Re-targeted to the current voice (HH2) and a brand-new unrelated account (admin login is broken). Unrelated account now gets HTTP 403 — the voice-preview authorization bug (issue #13) is FIXED.</t>
+          <t>Needs the owner + an unrelated non-admin account (cross-account check), so it signs those in itself. Unrelated account now gets HTTP 403 for the owner's HH2 preview — issue #13 is FIXED.</t>
         </is>
       </c>
     </row>
@@ -2464,7 +2456,7 @@
           <t>home.spec.ts</t>
         </is>
       </c>
-      <c r="F16" s="12" t="inlineStr">
+      <c r="F16" s="11" t="inlineStr">
         <is>
           <t>Skipped</t>
         </is>
@@ -2501,7 +2493,7 @@
           <t>home.spec.ts</t>
         </is>
       </c>
-      <c r="F17" s="12" t="inlineStr">
+      <c r="F17" s="11" t="inlineStr">
         <is>
           <t>Skipped</t>
         </is>
@@ -3175,7 +3167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3229,7 +3221,7 @@
           <t>Mobile · Library / Home</t>
         </is>
       </c>
-      <c r="C2" s="13" t="inlineStr">
+      <c r="C2" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3261,7 +3253,7 @@
           <t>Mobile · Audiobooks</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="C3" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3293,7 +3285,7 @@
           <t>Backend · Narration queue</t>
         </is>
       </c>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3325,7 +3317,7 @@
           <t>Mobile · Audiobooks</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="13" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
@@ -3357,24 +3349,24 @@
           <t>Web · Test environment</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>Info</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>The admin test account can no longer sign in, blocking 4 admin-only web tests (Home as admin, PDF catalogue, PDF upload, PDF → narration E2E).</t>
+          <t>The old admin test account (admin@yourdomain.com) no longer signs in (401); the admin account is now admin@gmail.com.</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>admin account from MOBILE_TEST_ADMIN_EMAIL: UI "Invalid email or password"; POST /api/auth/login → 401 (2026-10-02).</t>
+          <t>Switched to the new admin account on 2026-10-02; all 4 admin-only tests pass.</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>Needs new credentials</t>
+          <t>Resolved</t>
         </is>
       </c>
     </row>
@@ -3389,7 +3381,7 @@
           <t>Web · Security</t>
         </is>
       </c>
-      <c r="C7" s="15" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3421,7 +3413,7 @@
           <t>Web · Sign-in / sign-up</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
@@ -3453,7 +3445,7 @@
           <t>Web · Profile</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
@@ -3474,8 +3466,72 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>F-09</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Web · Auth (session)</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>The sign-in is an in-memory access token plus an httpOnly refresh cookie that rotates on use — replaying an older refresh cookie signs the browser out.</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Found while sharing one sign-in across the run; the test session helper now always carries the latest cookie.</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Not a bug (good practice)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>F-10</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Web · Admin account</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>The admin account shows "Confirm your email address" on every page (admin@gmail.com is unconfirmed).</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Banner seen on Voices / narration pages, 2026-10-02.</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Open — confirm the admin email</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F9"/>
+  <autoFilter ref="A1:F11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Odiobuk web: tests for develop's new features (TC-016..TC-024), final report
Grounded in AiSolutionsUSA/Audiobook origin/develop (2026-10-02) frontend:
- account-recovery.spec: forgot password (no account enumeration), reset
  link without token, email-confirm link missing/bogus token, show-password
  toggle — public pages, no sign-in, no email to a real person
- registration.spec: TC-001's new account also covers the welcome choice
  (TC-020), the Free-plan daily allowance on the narration page (TC-021),
  the confirm-email banner (TC-022) and empty Saved (TC-007)
- plans.spec: Free/Premium cards, invalid access code refused (TC-023)
- profile.spec: default speed + audiobook-ready email persist, restored (TC-024)
- Report: web 26/26 pass, mobile 33 pass + 2 skipped, 11 findings
</commit_message>
<xml_diff>
--- a/docs/odiobuk/Odiobuk_Test_Report.xlsx
+++ b/docs/odiobuk/Odiobuk_Test_Report.xlsx
@@ -13,9 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Web Results'!$A$1:$H$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Web Results'!$A$1:$H$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Mobile Results'!$A$1:$G$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Findings'!$A$1:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Findings'!$A$1:$F$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -595,10 +595,10 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="D7" s="5" t="n">
         <v>0</v>
@@ -618,14 +618,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Registration</t>
+          <t xml:space="preserve">   Registration &amp; first run</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D8" s="7" t="n">
         <v>0</v>
@@ -784,10 +784,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D14" s="7" t="n">
         <v>0</v>
@@ -861,52 +861,52 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Security</t>
+          <t xml:space="preserve">   Account recovery (signed out)</t>
         </is>
       </c>
       <c r="B17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Plans &amp; Premium</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
         <v>1</v>
       </c>
-      <c r="C17" s="6" t="n">
+      <c r="C18" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>MOBILE</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="n">
-        <v>35</v>
-      </c>
-      <c r="C18" s="4" t="n">
-        <v>33</v>
-      </c>
-      <c r="D18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="D18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
@@ -915,14 +915,14 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Login</t>
+          <t xml:space="preserve">   Security</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D19" s="7" t="n">
         <v>0</v>
@@ -940,27 +940,27 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Registration</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>4</v>
-      </c>
-      <c r="C20" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>MOBILE</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
@@ -969,14 +969,14 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Verified session</t>
+          <t xml:space="preserve">   Login</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C21" s="6" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D21" s="7" t="n">
         <v>0</v>
@@ -996,11 +996,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Home</t>
+          <t xml:space="preserve">   Registration</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C22" s="6" t="n">
         <v>4</v>
@@ -1012,7 +1012,7 @@
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1023,14 +1023,14 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Library</t>
+          <t xml:space="preserve">   Verified session</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C23" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D23" s="7" t="n">
         <v>0</v>
@@ -1050,14 +1050,14 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Audiobooks &amp; Player</t>
+          <t xml:space="preserve">   Home</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C24" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D24" s="7" t="n">
         <v>0</v>
@@ -1066,7 +1066,7 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1077,14 +1077,14 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Voices</t>
+          <t xml:space="preserve">   Library</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C25" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D25" s="7" t="n">
         <v>0</v>
@@ -1104,14 +1104,14 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Profile</t>
+          <t xml:space="preserve">   Audiobooks &amp; Player</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C26" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D26" s="7" t="n">
         <v>0</v>
@@ -1131,52 +1131,79 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Voices</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>5</v>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Profile</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>4</v>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t xml:space="preserve">   Vault</t>
         </is>
       </c>
-      <c r="B27" t="n">
+      <c r="B29" t="n">
         <v>2</v>
       </c>
-      <c r="C27" s="6" t="n">
+      <c r="C29" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="D27" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL (web + mobile)</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="n">
-        <v>52</v>
-      </c>
-      <c r="C28" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="D28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G28" s="3" t="inlineStr">
+      <c r="D29" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
@@ -1185,7 +1212,34 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Findings: 10 (see the Findings sheet)</t>
+          <t>TOTAL (web + mobile)</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>61</v>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Findings: 11 (see the Findings sheet)</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1263,7 +1317,7 @@
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Registration &amp; first run</t>
         </is>
       </c>
       <c r="C2" s="9" t="inlineStr">
@@ -1287,7 +1341,7 @@
         </is>
       </c>
       <c r="G2" s="9" t="n">
-        <v>11.2</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H2" s="9" t="inlineStr">
         <is>
@@ -1543,7 +1597,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Registration</t>
+          <t>Registration &amp; first run</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -1567,7 +1621,7 @@
         </is>
       </c>
       <c r="G9" s="9" t="n">
-        <v>5.6</v>
+        <v>4.5</v>
       </c>
       <c r="H9" s="9" t="inlineStr">
         <is>
@@ -1898,45 +1952,405 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
+          <t>TC-016</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Account recovery (signed out)</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Forgot password answers the same whether or not the account exists</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>New feature</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>account-recovery.spec.ts</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>NEW (develop feature). Public page, no sign-in. Unregistered address → neutral "Check your email" (no account enumeration); no email goes to a real person.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>TC-017</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Account recovery (signed out)</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Reset password without a token offers to request a new link</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>New feature</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>account-recovery.spec.ts</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>NEW (develop feature). Public page. No token → "Request a new link", no password form.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>TC-018</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Account recovery (signed out)</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Email confirmation link without a valid token is refused with a way forward</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>New feature</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>account-recovery.spec.ts</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>NEW (develop feature). Public page. Missing token → "missing its token" + "Send a new link"; bogus token → invalid/expired.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>TC-019</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Account recovery (signed out)</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Sign-in password field can be shown and hidden</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>New feature</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>account-recovery.spec.ts</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>NEW (develop feature). Public page. Show-password toggle flips aria-pressed and the input type, both ways.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>TC-020</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Registration &amp; first run</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Welcome: choosing "Listen to audiobooks" lands on the Library</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>New feature</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>registration.spec.ts</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>NEW (develop feature). On TC-001's new account: Continue with no choice is refused; "Listen to audiobooks" → Library.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>TC-021</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Registration &amp; first run</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Narration page explains the Free plan daily allowance before generating</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>New feature</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>registration.spec.ts</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>NEW (develop feature). On TC-001's new Free account (staff never see it): "Today: N of M audiobooks · up to X characters each" + "Premium allows more a day →". Nothing generated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>TC-022</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Registration &amp; first run</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Unconfirmed account sees the "Confirm your email" banner and can hide it</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>New feature</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>registration.spec.ts</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>NEW (develop feature). On TC-001's new unconfirmed account. "Resend link" deliberately not clicked (would send real email).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>TC-023</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Plans &amp; Premium</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Plans lists Free and Premium, and an invalid access code is refused</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>New feature</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>plans.spec.ts</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="H25" s="9" t="inlineStr">
+        <is>
+          <t>NEW (develop feature). Shared session (the run's single admin sign-in). Free + Premium cards with server-worded perks; empty and made-up codes refused; plan unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>TC-024</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Profile (You)</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Default playback speed and the "audiobook ready" email setting are saved</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>New feature</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>profile.spec.ts</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>NEW (develop feature). Shared session (the run's single admin sign-in). Speed + "audiobook ready" email both persist across reload, then restored. First attempt failed on a test issue (the checkbox flips only after the server saves); fixed and re-run alone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
           <t>SEC-001</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C27" s="9" t="inlineStr">
         <is>
           <t>An unrelated account should not be able to fetch another user's voice preview by guessing its id</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E27" s="9" t="inlineStr">
         <is>
           <t>voice-privacy-security.spec.ts</t>
         </is>
       </c>
-      <c r="F18" s="10" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="G18" s="9" t="n">
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="n">
         <v>27</v>
       </c>
-      <c r="H18" s="9" t="inlineStr">
+      <c r="H27" s="9" t="inlineStr">
         <is>
           <t>Needs the owner + an unrelated non-admin account (cross-account check), so it signs those in itself. Unrelated account now gets HTTP 403 for the owner's HH2 preview — issue #13 is FIXED.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H18"/>
+  <autoFilter ref="A1:H27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3167,7 +3581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3501,37 +3915,69 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
+          <t>F-11</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Web · New features (develop, 2026-10-02)</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Live site already runs develop's new features: password reset, email confirmation + banner, show-password, welcome step, Plans/Premium by access code, Free-plan daily allowance (2/day, 500 chars; Premium 5/day, 1,000 chars; one at a time), default speed and audiobook-ready email settings.</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>9 new tests TC-016…TC-024, all pass. Staff/admin accounts are exempt from the daily allowance (not shown).</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Covered</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
           <t>F-10</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Web · Admin account</t>
         </is>
       </c>
-      <c r="C11" s="15" t="inlineStr">
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>The admin account shows "Confirm your email address" on every page (admin@gmail.com is unconfirmed).</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E12" s="9" t="inlineStr">
         <is>
           <t>Banner seen on Voices / narration pages, 2026-10-02.</t>
         </is>
       </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>Open — confirm the admin email</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F11"/>
+  <autoFilter ref="A1:F12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>